<commit_message>
feat: add 8 new members to Engineer's Day 2026 QR registry and certificates (46 total)
</commit_message>
<xml_diff>
--- a/JNTUGV_Engineers_Day_2026_Certificates_QR.xlsx
+++ b/JNTUGV_Engineers_Day_2026_Certificates_QR.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,6 +42,11 @@
       <b val="1"/>
       <color rgb="000F172A"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="00475569"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Consolas"/>
@@ -114,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -135,9 +140,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -220,7 +228,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
@@ -245,7 +253,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>4</row>
       <rowOff>0</rowOff>
@@ -270,7 +278,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>5</row>
       <rowOff>0</rowOff>
@@ -295,7 +303,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>6</row>
       <rowOff>0</rowOff>
@@ -320,7 +328,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>7</row>
       <rowOff>0</rowOff>
@@ -345,7 +353,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>8</row>
       <rowOff>0</rowOff>
@@ -370,7 +378,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>9</row>
       <rowOff>0</rowOff>
@@ -395,7 +403,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>10</row>
       <rowOff>0</rowOff>
@@ -420,7 +428,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>11</row>
       <rowOff>0</rowOff>
@@ -445,7 +453,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>12</row>
       <rowOff>0</rowOff>
@@ -470,7 +478,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>13</row>
       <rowOff>0</rowOff>
@@ -495,7 +503,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>14</row>
       <rowOff>0</rowOff>
@@ -520,7 +528,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>15</row>
       <rowOff>0</rowOff>
@@ -545,7 +553,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>16</row>
       <rowOff>0</rowOff>
@@ -570,7 +578,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>17</row>
       <rowOff>0</rowOff>
@@ -595,7 +603,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>18</row>
       <rowOff>0</rowOff>
@@ -620,7 +628,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>19</row>
       <rowOff>0</rowOff>
@@ -645,7 +653,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>20</row>
       <rowOff>0</rowOff>
@@ -670,7 +678,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>21</row>
       <rowOff>0</rowOff>
@@ -695,7 +703,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>22</row>
       <rowOff>0</rowOff>
@@ -720,7 +728,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>23</row>
       <rowOff>0</rowOff>
@@ -745,7 +753,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>24</row>
       <rowOff>0</rowOff>
@@ -770,7 +778,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>25</row>
       <rowOff>0</rowOff>
@@ -795,7 +803,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>26</row>
       <rowOff>0</rowOff>
@@ -820,7 +828,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>27</row>
       <rowOff>0</rowOff>
@@ -845,7 +853,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>28</row>
       <rowOff>0</rowOff>
@@ -870,7 +878,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>29</row>
       <rowOff>0</rowOff>
@@ -895,7 +903,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>30</row>
       <rowOff>0</rowOff>
@@ -920,7 +928,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>31</row>
       <rowOff>0</rowOff>
@@ -945,7 +953,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>32</row>
       <rowOff>0</rowOff>
@@ -970,7 +978,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>33</row>
       <rowOff>0</rowOff>
@@ -995,7 +1003,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>34</row>
       <rowOff>0</rowOff>
@@ -1020,7 +1028,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>35</row>
       <rowOff>0</rowOff>
@@ -1045,7 +1053,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>36</row>
       <rowOff>0</rowOff>
@@ -1070,7 +1078,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>37</row>
       <rowOff>0</rowOff>
@@ -1095,7 +1103,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>38</row>
       <rowOff>0</rowOff>
@@ -1120,7 +1128,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>39</row>
       <rowOff>0</rowOff>
@@ -1145,7 +1153,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>40</row>
       <rowOff>0</rowOff>
@@ -1158,6 +1166,206 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId38"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId39"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>42</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId40"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>43</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId41"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>44</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId42"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId43"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>46</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId44"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>47</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="45" name="Image 45" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId45"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>48</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="46" name="Image 46" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId46"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1460,15 +1668,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="65" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1481,7 +1690,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>National Engineer's Day 2026 • Summer Internship Certificate QR Registry</t>
+          <t>National Engineer's Day 2026 • Summer Internship Certificate QR Registry (46 Members)</t>
         </is>
       </c>
     </row>
@@ -1498,20 +1707,25 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
+          <t>Roll / Reg No</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
           <t>Certificate ID</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Verification URL (Click to Open)</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>QR Preview</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -1528,16 +1742,21 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-001</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-001</t>
         </is>
       </c>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -1554,16 +1773,21 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-002</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-002</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -1580,16 +1804,21 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-003</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-003</t>
         </is>
       </c>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -1606,16 +1835,21 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-004</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-004</t>
         </is>
       </c>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -1632,16 +1866,21 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-005</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-005</t>
         </is>
       </c>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -1658,16 +1897,21 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-006</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-006</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n"/>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -1684,16 +1928,21 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-007</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-007</t>
         </is>
       </c>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -1710,16 +1959,21 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-008</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-008</t>
         </is>
       </c>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -1736,16 +1990,21 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-009</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-009</t>
         </is>
       </c>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="F12" s="4" t="n"/>
+      <c r="G12" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -1762,16 +2021,21 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-010</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-010</t>
         </is>
       </c>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -1788,16 +2052,21 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-011</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-011</t>
         </is>
       </c>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="F14" s="4" t="n"/>
+      <c r="G14" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -1814,16 +2083,21 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-012</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-012</t>
         </is>
       </c>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="8" t="inlineStr">
+      <c r="F15" s="4" t="n"/>
+      <c r="G15" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -1840,16 +2114,21 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-013</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-013</t>
         </is>
       </c>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="F16" s="4" t="n"/>
+      <c r="G16" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -1866,16 +2145,21 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-014</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-014</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="F17" s="4" t="n"/>
+      <c r="G17" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -1892,16 +2176,21 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-015</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-015</t>
         </is>
       </c>
-      <c r="E18" s="4" t="n"/>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="F18" s="4" t="n"/>
+      <c r="G18" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -1918,16 +2207,21 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-016</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-016</t>
         </is>
       </c>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="8" t="inlineStr">
+      <c r="F19" s="4" t="n"/>
+      <c r="G19" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -1944,16 +2238,21 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-017</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-017</t>
         </is>
       </c>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="F20" s="4" t="n"/>
+      <c r="G20" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -1970,16 +2269,21 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-018</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-018</t>
         </is>
       </c>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="8" t="inlineStr">
+      <c r="F21" s="4" t="n"/>
+      <c r="G21" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -1996,16 +2300,21 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-019</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-019</t>
         </is>
       </c>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2022,16 +2331,21 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-020</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-020</t>
         </is>
       </c>
-      <c r="E23" s="4" t="n"/>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="F23" s="4" t="n"/>
+      <c r="G23" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2048,16 +2362,21 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-021</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="E24" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-021</t>
         </is>
       </c>
-      <c r="E24" s="4" t="n"/>
-      <c r="F24" s="8" t="inlineStr">
+      <c r="F24" s="4" t="n"/>
+      <c r="G24" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2074,16 +2393,21 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-022</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-022</t>
         </is>
       </c>
-      <c r="E25" s="4" t="n"/>
-      <c r="F25" s="8" t="inlineStr">
+      <c r="F25" s="4" t="n"/>
+      <c r="G25" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2100,16 +2424,21 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-023</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="E26" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-023</t>
         </is>
       </c>
-      <c r="E26" s="4" t="n"/>
-      <c r="F26" s="8" t="inlineStr">
+      <c r="F26" s="4" t="n"/>
+      <c r="G26" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2126,16 +2455,21 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-024</t>
         </is>
       </c>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-024</t>
         </is>
       </c>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="8" t="inlineStr">
+      <c r="F27" s="4" t="n"/>
+      <c r="G27" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2152,16 +2486,21 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-025</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="E28" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-025</t>
         </is>
       </c>
-      <c r="E28" s="4" t="n"/>
-      <c r="F28" s="8" t="inlineStr">
+      <c r="F28" s="4" t="n"/>
+      <c r="G28" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2178,16 +2517,21 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-026</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="E29" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-026</t>
         </is>
       </c>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="8" t="inlineStr">
+      <c r="F29" s="4" t="n"/>
+      <c r="G29" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2204,16 +2548,21 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-027</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="E30" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-027</t>
         </is>
       </c>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="8" t="inlineStr">
+      <c r="F30" s="4" t="n"/>
+      <c r="G30" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2230,16 +2579,21 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-028</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="E31" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-028</t>
         </is>
       </c>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="8" t="inlineStr">
+      <c r="F31" s="4" t="n"/>
+      <c r="G31" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2256,16 +2610,21 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-029</t>
         </is>
       </c>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="E32" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-029</t>
         </is>
       </c>
-      <c r="E32" s="4" t="n"/>
-      <c r="F32" s="8" t="inlineStr">
+      <c r="F32" s="4" t="n"/>
+      <c r="G32" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2282,16 +2641,21 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-030</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="E33" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-030</t>
         </is>
       </c>
-      <c r="E33" s="4" t="n"/>
-      <c r="F33" s="8" t="inlineStr">
+      <c r="F33" s="4" t="n"/>
+      <c r="G33" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2308,16 +2672,21 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-031</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="E34" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-031</t>
         </is>
       </c>
-      <c r="E34" s="4" t="n"/>
-      <c r="F34" s="8" t="inlineStr">
+      <c r="F34" s="4" t="n"/>
+      <c r="G34" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2334,16 +2703,21 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-032</t>
         </is>
       </c>
-      <c r="D35" s="7" t="inlineStr">
+      <c r="E35" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-032</t>
         </is>
       </c>
-      <c r="E35" s="4" t="n"/>
-      <c r="F35" s="8" t="inlineStr">
+      <c r="F35" s="4" t="n"/>
+      <c r="G35" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2360,16 +2734,21 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-033</t>
         </is>
       </c>
-      <c r="D36" s="7" t="inlineStr">
+      <c r="E36" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-033</t>
         </is>
       </c>
-      <c r="E36" s="4" t="n"/>
-      <c r="F36" s="8" t="inlineStr">
+      <c r="F36" s="4" t="n"/>
+      <c r="G36" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2386,16 +2765,21 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-034</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="E37" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-034</t>
         </is>
       </c>
-      <c r="E37" s="4" t="n"/>
-      <c r="F37" s="8" t="inlineStr">
+      <c r="F37" s="4" t="n"/>
+      <c r="G37" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2412,16 +2796,21 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-035</t>
         </is>
       </c>
-      <c r="D38" s="7" t="inlineStr">
+      <c r="E38" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-035</t>
         </is>
       </c>
-      <c r="E38" s="4" t="n"/>
-      <c r="F38" s="8" t="inlineStr">
+      <c r="F38" s="4" t="n"/>
+      <c r="G38" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2438,16 +2827,21 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-036</t>
         </is>
       </c>
-      <c r="D39" s="7" t="inlineStr">
+      <c r="E39" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-036</t>
         </is>
       </c>
-      <c r="E39" s="4" t="n"/>
-      <c r="F39" s="8" t="inlineStr">
+      <c r="F39" s="4" t="n"/>
+      <c r="G39" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2464,16 +2858,21 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-037</t>
         </is>
       </c>
-      <c r="D40" s="7" t="inlineStr">
+      <c r="E40" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-037</t>
         </is>
       </c>
-      <c r="E40" s="4" t="n"/>
-      <c r="F40" s="8" t="inlineStr">
+      <c r="F40" s="4" t="n"/>
+      <c r="G40" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2490,16 +2889,269 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
           <t>JNTUGV-ED26-038</t>
         </is>
       </c>
-      <c r="D41" s="7" t="inlineStr">
+      <c r="E41" s="8" t="inlineStr">
         <is>
           <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-038</t>
         </is>
       </c>
-      <c r="E41" s="4" t="n"/>
-      <c r="F41" s="8" t="inlineStr">
+      <c r="F41" s="4" t="n"/>
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="70" customHeight="1">
+      <c r="A42" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>KOLATI SOWMYA SRI</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>23VV1A0109</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-039</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-039</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="n"/>
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="70" customHeight="1">
+      <c r="A43" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>KUNA CHANDRIIKA</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>23VV1A0110</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-040</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-040</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="n"/>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="70" customHeight="1">
+      <c r="A44" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Patarlapalli Meena</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>23VV1A0122</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-041</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-041</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="n"/>
+      <c r="G44" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="70" customHeight="1">
+      <c r="A45" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Pedapati Leela Sri Deepthi</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>23VV1A0123</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-042</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-042</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="n"/>
+      <c r="G45" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="70" customHeight="1">
+      <c r="A46" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Vanthala Dhanalakshmi</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>23VV1A0130</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-043</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-043</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="n"/>
+      <c r="G46" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="70" customHeight="1">
+      <c r="A47" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>GURUBELLU SIRISHA</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>24VV5A0135</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-044</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-044</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="n"/>
+      <c r="G47" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="70" customHeight="1">
+      <c r="A48" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Madaka Pavitra</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>24VV5A0136</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-045</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-045</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="n"/>
+      <c r="G48" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="70" customHeight="1">
+      <c r="A49" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Panchada Pushpa</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>24VV1A0137</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-046</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-046</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="n"/>
+      <c r="G49" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -2507,50 +3159,58 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId39"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId47"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add 9 new students (55 members total) with distinct QRs, Excel and registry
</commit_message>
<xml_diff>
--- a/JNTUGV_Engineers_Day_2026_Certificates_QR.xlsx
+++ b/JNTUGV_Engineers_Day_2026_Certificates_QR.xlsx
@@ -1366,6 +1366,231 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId46"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>49</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="47" name="Image 47" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId47"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>50</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="48" name="Image 48" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId48"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>51</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="49" name="Image 49" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId49"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>52</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="50" name="Image 50" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId50"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>53</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="51" name="Image 51" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId51"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>54</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="52" name="Image 52" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId52"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>55</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="53" name="Image 53" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId53"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>56</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="54" name="Image 54" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId54"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>57</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="55" name="Image 55" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId55"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1668,7 +1893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1690,7 +1915,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>National Engineer's Day 2026 • Summer Internship Certificate QR Registry (46 Members)</t>
+          <t>National Engineer's Day 2026 • Summer Internship Certificate QR Registry (55 Members)</t>
         </is>
       </c>
     </row>
@@ -3152,6 +3377,285 @@
       </c>
       <c r="F49" s="4" t="n"/>
       <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="70" customHeight="1">
+      <c r="A50" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>JONNALAGADDA PREM SAGAR</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-047</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-047</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="n"/>
+      <c r="G50" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="70" customHeight="1">
+      <c r="A51" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>BADAM LEELA AVINASH</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-048</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-048</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="n"/>
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="70" customHeight="1">
+      <c r="A52" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>SEELAM GOWRI CHARAN</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-049</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-049</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="n"/>
+      <c r="G52" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="70" customHeight="1">
+      <c r="A53" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>SIRINGI VINAY</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-050</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-050</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="n"/>
+      <c r="G53" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="70" customHeight="1">
+      <c r="A54" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>POLAVARAPU PHANI DURGA MANI SRINIVASA RAO</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-051</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-051</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="n"/>
+      <c r="G54" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="70" customHeight="1">
+      <c r="A55" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>KURA NARENDRA KUMAR</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-052</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-052</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="n"/>
+      <c r="G55" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="70" customHeight="1">
+      <c r="A56" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>RANGU SRAVYA</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-053</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-053</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="n"/>
+      <c r="G56" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="70" customHeight="1">
+      <c r="A57" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>PITHANI BHARGAVI SRI SATYA SRUJANA</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-054</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-054</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="n"/>
+      <c r="G57" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="70" customHeight="1">
+      <c r="A58" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>PINAKANA SNEHA SWAROOP</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-055</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-055</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="n"/>
+      <c r="G58" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -3209,8 +3713,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId47"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId56"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(certifications): configure direct QR redirects for team 47-49 and contributors 50-55 to CAP portal
</commit_message>
<xml_diff>
--- a/JNTUGV_Engineers_Day_2026_Certificates_QR.xlsx
+++ b/JNTUGV_Engineers_Day_2026_Certificates_QR.xlsx
@@ -3388,7 +3388,7 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>JONNALAGADDA PREM SAGAR</t>
+          <t>Jonnalagadda Prem Sagar</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -3403,7 +3403,7 @@
       </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-047</t>
+          <t>https://cap.jntugv.edu.in/about/team</t>
         </is>
       </c>
       <c r="F50" s="4" t="n"/>
@@ -3419,7 +3419,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>BADAM LEELA AVINASH</t>
+          <t>Badam Leela Avinash</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -3434,7 +3434,7 @@
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-048</t>
+          <t>https://cap.jntugv.edu.in/about/team</t>
         </is>
       </c>
       <c r="F51" s="4" t="n"/>
@@ -3450,7 +3450,7 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>SEELAM GOWRI CHARAN</t>
+          <t>Seelam Gowri Charan</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="E52" s="8" t="inlineStr">
         <is>
-          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-049</t>
+          <t>https://cap.jntugv.edu.in/about/team</t>
         </is>
       </c>
       <c r="F52" s="4" t="n"/>
@@ -3481,7 +3481,7 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>SIRINGI VINAY</t>
+          <t>Siringi Vinay</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
-          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-050</t>
+          <t>https://cap.jntugv.edu.in/contributors</t>
         </is>
       </c>
       <c r="F53" s="4" t="n"/>
@@ -3512,7 +3512,7 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>POLAVARAPU PHANI DURGA MANI SRINIVASA RAO</t>
+          <t>Polavarapu Phani Durga Mani Srinivasa Rao</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -3527,7 +3527,7 @@
       </c>
       <c r="E54" s="8" t="inlineStr">
         <is>
-          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-051</t>
+          <t>https://cap.jntugv.edu.in/contributors</t>
         </is>
       </c>
       <c r="F54" s="4" t="n"/>
@@ -3543,7 +3543,7 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>KURA NARENDRA KUMAR</t>
+          <t>Kura Narendra Kumar</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-052</t>
+          <t>https://cap.jntugv.edu.in/contributors</t>
         </is>
       </c>
       <c r="F55" s="4" t="n"/>
@@ -3574,7 +3574,7 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>RANGU SRAVYA</t>
+          <t>Rangu Sravya</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
@@ -3589,7 +3589,7 @@
       </c>
       <c r="E56" s="8" t="inlineStr">
         <is>
-          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-053</t>
+          <t>https://cap.jntugv.edu.in/contributors</t>
         </is>
       </c>
       <c r="F56" s="4" t="n"/>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>PITHANI BHARGAVI SRI SATYA SRUJANA</t>
+          <t>Pithani Bhargavi Sri Satya Srujana</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -3620,7 +3620,7 @@
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-054</t>
+          <t>https://cap.jntugv.edu.in/contributors</t>
         </is>
       </c>
       <c r="F57" s="4" t="n"/>
@@ -3636,7 +3636,7 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>PINAKANA SNEHA SWAROOP</t>
+          <t>Pinakana Sneha Swaroop</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -3651,7 +3651,7 @@
       </c>
       <c r="E58" s="8" t="inlineStr">
         <is>
-          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-055</t>
+          <t>https://cap.jntugv.edu.in/contributors</t>
         </is>
       </c>
       <c r="F58" s="4" t="n"/>

</xml_diff>

<commit_message>
feat(certifications): add 4 new members (Chidwilash, G Dhana Sai, Vinay D, Mohan S) with QR codes and registry entries
</commit_message>
<xml_diff>
--- a/JNTUGV_Engineers_Day_2026_Certificates_QR.xlsx
+++ b/JNTUGV_Engineers_Day_2026_Certificates_QR.xlsx
@@ -1591,6 +1591,106 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId55"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>58</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="56" name="Image 56" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId56"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>59</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="57" name="Image 57" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId57"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>60</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="58" name="Image 58" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId58"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>61</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="59" name="Image 59" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId59"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1893,7 +1993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3656,6 +3756,130 @@
       </c>
       <c r="F58" s="4" t="n"/>
       <c r="G58" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="70" customHeight="1">
+      <c r="A59" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Chidwilash</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-056</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-056</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="n"/>
+      <c r="G59" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="70" customHeight="1">
+      <c r="A60" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>G Dhana Sai</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-057</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-057</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="n"/>
+      <c r="G60" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="70" customHeight="1">
+      <c r="A61" s="4" t="n">
+        <v>58</v>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Vinay D</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-058</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-058</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="n"/>
+      <c r="G61" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="70" customHeight="1">
+      <c r="A62" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Mohan S</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>JNTUGV-ED26-059</t>
+        </is>
+      </c>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>https://jntugvcev.edu.in/engineersday2026/certifications?id=JNTUGV-ED26-059</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="n"/>
+      <c r="G62" s="9" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -3722,8 +3946,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId59"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId56"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId60"/>
 </worksheet>
 </file>
</xml_diff>